<commit_message>
Add program guidance and detection examples
</commit_message>
<xml_diff>
--- a/Maturity Matrix/Maturity_Matrix.xlsx
+++ b/Maturity Matrix/Maturity_Matrix.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rb3a6c7f89c184f09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R754697af27334805"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Guide" sheetId="2" r:id="R4abc61ee63f84fe4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -145,7 +146,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="4">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="12"/>
       <x:color theme="1"/>
@@ -153,23 +154,34 @@
     </x:font>
     <x:font>
       <x:sz val="11"/>
-      <x:color rgb="1F2933"/>
+      <x:color rgb="FF1F2933"/>
       <x:name val="Calibri"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="102A43"/>
+      <x:color rgb="FF102A43"/>
       <x:name val="Calibri"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="1F2933"/>
+      <x:color rgb="FF1F2933"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2933"/>
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -178,46 +190,76 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="D9EAF7"/>
+        <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFF"/>
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="D9EAF7"/>
+        <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFF"/>
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="D9EAF7"/>
+        <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFF"/>
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="D9EAF7"/>
+        <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFF"/>
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="4">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -235,23 +277,37 @@
     </x:border>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="D9E2EC"/>
+        <x:color rgb="FFD9E2EC"/>
       </x:left>
       <x:right style="thin">
-        <x:color rgb="D9E2EC"/>
+        <x:color rgb="FFD9E2EC"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="D9E2EC"/>
+        <x:color rgb="FFD9E2EC"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="D9E2EC"/>
+        <x:color rgb="FFD9E2EC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB8C7D9"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB8C7D9"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB8C7D9"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB8C7D9"/>
       </x:bottom>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="32">
+  <x:cellXfs count="48">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -339,6 +395,40 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -923,4 +1013,338 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="33.33000183105469" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="33.33000183105469" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="26.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28.889999389648438" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="46" t="str">
+        <x:v>Insider Threat Program Maturity Scoring Guide</x:v>
+      </x:c>
+      <x:c r="B1" s="46"/>
+      <x:c r="C1" s="46"/>
+      <x:c r="D1" s="46"/>
+      <x:c r="E1" s="46"/>
+      <x:c r="F1" s="46"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="47" t="str">
+        <x:v>Score</x:v>
+      </x:c>
+      <x:c r="B3" s="47" t="str">
+        <x:v>Stage</x:v>
+      </x:c>
+      <x:c r="C3" s="47" t="str">
+        <x:v>Definition</x:v>
+      </x:c>
+      <x:c r="D3" s="47" t="str">
+        <x:v>Evidence Examples</x:v>
+      </x:c>
+      <x:c r="E3" s="47" t="str">
+        <x:v>Use When</x:v>
+      </x:c>
+      <x:c r="F3" s="47" t="str">
+        <x:v>Action</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="43" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B4" s="43" t="str">
+        <x:v>Initial</x:v>
+      </x:c>
+      <x:c r="C4" s="43" t="str">
+        <x:v>General awareness exists, but no repeatable capability is in place.</x:v>
+      </x:c>
+      <x:c r="D4" s="43" t="str">
+        <x:v>No documented owner, process, telemetry, or detection.</x:v>
+      </x:c>
+      <x:c r="E4" s="43" t="str">
+        <x:v>The area is known but unmanaged.</x:v>
+      </x:c>
+      <x:c r="F4" s="43" t="str">
+        <x:v>Assign ownership and define minimum requirements.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="43" t="str">
+        <x:v>Minimal</x:v>
+      </x:c>
+      <x:c r="C5" s="43" t="str">
+        <x:v>Basic activity exists to meet an initial requirement.</x:v>
+      </x:c>
+      <x:c r="D5" s="43" t="str">
+        <x:v>Ad hoc process, partial telemetry, limited documentation.</x:v>
+      </x:c>
+      <x:c r="E5" s="43" t="str">
+        <x:v>Coverage exists but depends on individual effort.</x:v>
+      </x:c>
+      <x:c r="F5" s="43" t="str">
+        <x:v>Document process and identify required data sources.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="43" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="43" t="str">
+        <x:v>Procedural</x:v>
+      </x:c>
+      <x:c r="C6" s="43" t="str">
+        <x:v>Process is defined and repeatable.</x:v>
+      </x:c>
+      <x:c r="D6" s="43" t="str">
+        <x:v>Documented workflow, periodic review, basic alert handling.</x:v>
+      </x:c>
+      <x:c r="E6" s="43" t="str">
+        <x:v>The area exceeds minimum requirements.</x:v>
+      </x:c>
+      <x:c r="F6" s="43" t="str">
+        <x:v>Add tuning, quality review, and stakeholder review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="43" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="43" t="str">
+        <x:v>Innovative</x:v>
+      </x:c>
+      <x:c r="C7" s="43" t="str">
+        <x:v>Capability is established and actively improved.</x:v>
+      </x:c>
+      <x:c r="D7" s="43" t="str">
+        <x:v>Correlated detections, risk context, testing, metrics.</x:v>
+      </x:c>
+      <x:c r="E7" s="43" t="str">
+        <x:v>The area is mature and improving.</x:v>
+      </x:c>
+      <x:c r="F7" s="43" t="str">
+        <x:v>Automate correlation and response where appropriate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="43" t="str">
+        <x:v>Leading</x:v>
+      </x:c>
+      <x:c r="C8" s="43" t="str">
+        <x:v>Capability is mature, measured, and maintained.</x:v>
+      </x:c>
+      <x:c r="D8" s="43" t="str">
+        <x:v>Documented ownership, tested controls, metrics, continuous improvement.</x:v>
+      </x:c>
+      <x:c r="E8" s="43" t="str">
+        <x:v>Only routine maintenance is needed.</x:v>
+      </x:c>
+      <x:c r="F8" s="43" t="str">
+        <x:v>Review for changes in business, tools, and threat landscape.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="47" t="str">
+        <x:v>Suggested Assessment Workflow</x:v>
+      </x:c>
+      <x:c r="B10" s="47"/>
+      <x:c r="C10" s="47"/>
+      <x:c r="D10" s="47"/>
+      <x:c r="E10" s="47"/>
+      <x:c r="F10" s="47"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="43" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B11" s="43" t="str">
+        <x:v>Scope</x:v>
+      </x:c>
+      <x:c r="C11" s="43" t="str">
+        <x:v>Select business units, data types, and employee populations.</x:v>
+      </x:c>
+      <x:c r="D11" s="43" t="str"/>
+      <x:c r="E11" s="43" t="str"/>
+      <x:c r="F11" s="43" t="str"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="43" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B12" s="43" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="C12" s="43" t="str">
+        <x:v>Collect process documents, telemetry proof, detection examples, and response records.</x:v>
+      </x:c>
+      <x:c r="D12" s="43" t="str"/>
+      <x:c r="E12" s="43" t="str"/>
+      <x:c r="F12" s="43" t="str"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="43" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B13" s="43" t="str">
+        <x:v>Score</x:v>
+      </x:c>
+      <x:c r="C13" s="43" t="str">
+        <x:v>Assign 0-4 for each row in the main matrix based on evidence.</x:v>
+      </x:c>
+      <x:c r="D13" s="43" t="str"/>
+      <x:c r="E13" s="43" t="str"/>
+      <x:c r="F13" s="43" t="str"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="43" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B14" s="43" t="str">
+        <x:v>Prioritize</x:v>
+      </x:c>
+      <x:c r="C14" s="43" t="str">
+        <x:v>Focus first on high-risk rows with low maturity and available telemetry.</x:v>
+      </x:c>
+      <x:c r="D14" s="43" t="str"/>
+      <x:c r="E14" s="43" t="str"/>
+      <x:c r="F14" s="43" t="str"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="43" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B15" s="43" t="str">
+        <x:v>Improve</x:v>
+      </x:c>
+      <x:c r="C15" s="43" t="str">
+        <x:v>Create owners, data-source tasks, detection work, and response playbooks.</x:v>
+      </x:c>
+      <x:c r="D15" s="43" t="str"/>
+      <x:c r="E15" s="43" t="str"/>
+      <x:c r="F15" s="43" t="str"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="43" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B16" s="43" t="str">
+        <x:v>Review</x:v>
+      </x:c>
+      <x:c r="C16" s="43" t="str">
+        <x:v>Re-score quarterly or after major organizational, tooling, or regulatory changes.</x:v>
+      </x:c>
+      <x:c r="D16" s="43" t="str"/>
+      <x:c r="E16" s="43" t="str"/>
+      <x:c r="F16" s="43" t="str"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="47" t="str">
+        <x:v>Recommended Evidence Fields</x:v>
+      </x:c>
+      <x:c r="B18" s="47"/>
+      <x:c r="C18" s="47"/>
+      <x:c r="D18" s="47"/>
+      <x:c r="E18" s="47"/>
+      <x:c r="F18" s="47"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="43" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="B19" s="43" t="str">
+        <x:v>Named team or role accountable for the capability.</x:v>
+      </x:c>
+      <x:c r="C19" s="43" t="str"/>
+      <x:c r="D19" s="43" t="str"/>
+      <x:c r="E19" s="43" t="str"/>
+      <x:c r="F19" s="43" t="str"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="43" t="str">
+        <x:v>Telemetry</x:v>
+      </x:c>
+      <x:c r="B20" s="43" t="str">
+        <x:v>Log sources, data quality, retention, and coverage.</x:v>
+      </x:c>
+      <x:c r="C20" s="43" t="str"/>
+      <x:c r="D20" s="43" t="str"/>
+      <x:c r="E20" s="43" t="str"/>
+      <x:c r="F20" s="43" t="str"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="43" t="str">
+        <x:v>Detection</x:v>
+      </x:c>
+      <x:c r="B21" s="43" t="str">
+        <x:v>Alert logic, thresholds, false positives, and testing history.</x:v>
+      </x:c>
+      <x:c r="C21" s="43" t="str"/>
+      <x:c r="D21" s="43" t="str"/>
+      <x:c r="E21" s="43" t="str"/>
+      <x:c r="F21" s="43" t="str"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="43" t="str">
+        <x:v>Response</x:v>
+      </x:c>
+      <x:c r="B22" s="43" t="str">
+        <x:v>Escalation path, case handling, and decision records.</x:v>
+      </x:c>
+      <x:c r="C22" s="43" t="str"/>
+      <x:c r="D22" s="43" t="str"/>
+      <x:c r="E22" s="43" t="str"/>
+      <x:c r="F22" s="43" t="str"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="43" t="str">
+        <x:v>Governance</x:v>
+      </x:c>
+      <x:c r="B23" s="43" t="str">
+        <x:v>Legal, HR, privacy, and business approvals where needed.</x:v>
+      </x:c>
+      <x:c r="C23" s="43" t="str"/>
+      <x:c r="D23" s="43" t="str"/>
+      <x:c r="E23" s="43" t="str"/>
+      <x:c r="F23" s="43" t="str"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="43" t="str">
+        <x:v>Metrics</x:v>
+      </x:c>
+      <x:c r="B24" s="43" t="str">
+        <x:v>Alert volume, true positive rate, coverage, and review cadence.</x:v>
+      </x:c>
+      <x:c r="C24" s="43" t="str"/>
+      <x:c r="D24" s="43" t="str"/>
+      <x:c r="E24" s="43" t="str"/>
+      <x:c r="F24" s="43" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A10:F10"/>
+    <x:mergeCell ref="A18:F18"/>
+    <x:mergeCell ref="B19:F19"/>
+    <x:mergeCell ref="B20:F20"/>
+    <x:mergeCell ref="B21:F21"/>
+    <x:mergeCell ref="B22:F22"/>
+    <x:mergeCell ref="B23:F23"/>
+    <x:mergeCell ref="B24:F24"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>